<commit_message>
atualizando euclides da cunha e pojuca
</commit_message>
<xml_diff>
--- a/proposta_regionais_nova_regional.xlsx
+++ b/proposta_regionais_nova_regional.xlsx
@@ -1345,7 +1345,7 @@
     <t>LUÍS EDUARDO MAGALHÃES</t>
   </si>
   <si>
-    <t>NOVA_REGIONAL</t>
+    <t>NOVA REGIONAL</t>
   </si>
   <si>
     <t>RMS</t>
@@ -4653,7 +4653,7 @@
         <v>9</v>
       </c>
       <c r="F128" t="s">
-        <v>443</v>
+        <v>9</v>
       </c>
       <c r="G128" t="s">
         <v>446</v>
@@ -8839,10 +8839,10 @@
         <v>440</v>
       </c>
       <c r="F310" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G310" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="311" spans="1:7">

</xml_diff>